<commit_message>
Update Precio y Sabores de Bolis.xlsx
</commit_message>
<xml_diff>
--- a/datos/Precio y Sabores de Bolis.xlsx
+++ b/datos/Precio y Sabores de Bolis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pagina Venta Bolis\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A410361-ADEE-4041-A3CE-BCA1A67CAC6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5501691-9149-4FEF-BB0C-AD89CD1FDCBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="695" xr2:uid="{C9F31BEF-597D-471C-872A-5048C5703FC4}"/>
   </bookViews>
@@ -666,7 +666,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -710,7 +710,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="3" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -725,6 +724,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -746,7 +746,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -1071,27 +1070,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB2EAEE6-23BA-467B-8FCC-6B86426A06BE}">
-  <dimension ref="A1:T137"/>
+  <dimension ref="A1:Q137"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="27" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="46" t="s">
         <v>16</v>
       </c>
@@ -1100,17 +1096,16 @@
       <c r="D1" s="47"/>
       <c r="E1" s="47"/>
       <c r="F1" s="48"/>
-      <c r="G1" s="2"/>
-      <c r="K1" s="50" t="s">
+      <c r="H1" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="L1" s="51"/>
-      <c r="M1" s="51"/>
-      <c r="N1" s="51"/>
-      <c r="O1" s="52"/>
-      <c r="T1" s="1"/>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
+      <c r="K1" s="51"/>
+      <c r="L1" s="52"/>
+      <c r="Q1" s="1"/>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>49</v>
       </c>
@@ -1129,29 +1124,29 @@
       <c r="F2" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="K2" s="16" t="s">
+      <c r="H2" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="L2" s="17" t="s">
+      <c r="I2" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="17" t="s">
+      <c r="J2" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="N2" s="18" t="s">
+      <c r="K2" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="O2" s="19" t="s">
+      <c r="L2" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="P2" t="s">
+      <c r="M2" t="s">
         <v>55</v>
       </c>
-      <c r="T2" s="1"/>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="Q2" s="1"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="str">
-        <f>K3</f>
+        <f>H3</f>
         <v>Leche entera</v>
       </c>
       <c r="B3" s="27">
@@ -1164,34 +1159,34 @@
         <v>40</v>
       </c>
       <c r="E3" s="21">
-        <f>N3</f>
+        <f>K3</f>
         <v>30</v>
       </c>
       <c r="F3" s="24">
         <f>E3*B3</f>
         <v>30</v>
       </c>
-      <c r="J3">
+      <c r="G3">
         <v>1</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="L3" s="7">
+      <c r="I3" s="7">
         <v>1.5</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="J3" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="N3" s="8">
+      <c r="K3" s="8">
         <v>30</v>
       </c>
-      <c r="O3" s="10"/>
-      <c r="T3" s="1"/>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="L3" s="10"/>
+      <c r="Q3" s="1"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="str">
-        <f>K7</f>
+        <f>H7</f>
         <v>Vainilla</v>
       </c>
       <c r="B4" s="27">
@@ -1204,119 +1199,119 @@
         <v>40</v>
       </c>
       <c r="E4" s="21">
-        <f>N7</f>
+        <f>K7</f>
         <v>18.5</v>
       </c>
       <c r="F4" s="24">
-        <f>(N7/L7)*C4</f>
+        <f>(K7/I7)*C4</f>
         <v>3.7</v>
       </c>
-      <c r="J4">
-        <f>J3+1</f>
+      <c r="G4">
+        <f>G3+1</f>
         <v>2</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="H4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="L4" s="7">
+      <c r="I4" s="7">
         <v>180</v>
       </c>
-      <c r="M4" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="N4" s="8">
+      <c r="J4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="8">
         <v>58</v>
       </c>
-      <c r="O4" s="10"/>
-      <c r="T4" s="1"/>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="L4" s="10"/>
+      <c r="Q4" s="1"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="str">
-        <f>K4</f>
+        <f>H4</f>
         <v>CMC</v>
       </c>
       <c r="B5" s="27">
         <v>7.5</v>
       </c>
       <c r="C5" s="7">
-        <f>L4</f>
+        <f>I4</f>
         <v>180</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E5" s="21">
-        <f>N4</f>
+        <f>K4</f>
         <v>58</v>
       </c>
       <c r="F5" s="24">
         <f>(E5/C5)*B5</f>
         <v>2.416666666666667</v>
       </c>
-      <c r="J5">
-        <f t="shared" ref="J5:J24" si="0">J4+1</f>
+      <c r="G5">
+        <f t="shared" ref="G5:G24" si="0">G4+1</f>
         <v>3</v>
       </c>
-      <c r="K5" s="9" t="s">
+      <c r="H5" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="L5" s="7">
+      <c r="I5" s="7">
         <v>380</v>
       </c>
-      <c r="M5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="N5" s="8">
+      <c r="J5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K5" s="8">
         <v>29</v>
       </c>
-      <c r="O5" s="11">
+      <c r="L5" s="11">
         <v>20</v>
       </c>
-      <c r="T5" s="1"/>
-    </row>
-    <row r="6" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q5" s="1"/>
+    </row>
+    <row r="6" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="32" t="str">
-        <f>K5</f>
+        <f>H5</f>
         <v>Leche condensada</v>
       </c>
       <c r="B6" s="33">
         <v>1.5</v>
       </c>
       <c r="C6" s="34">
-        <f>L5</f>
+        <f>I5</f>
         <v>380</v>
       </c>
       <c r="D6" s="34" t="s">
         <v>13</v>
       </c>
       <c r="E6" s="35">
-        <f>N5</f>
+        <f>K5</f>
         <v>29</v>
       </c>
       <c r="F6" s="24">
         <f>E6*B6</f>
         <v>43.5</v>
       </c>
-      <c r="J6">
+      <c r="G6">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="K6" s="9" t="s">
+      <c r="H6" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="L6" s="7">
+      <c r="I6" s="7">
         <v>1</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="J6" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="N6" s="8">
+      <c r="K6" s="8">
         <v>60</v>
       </c>
-      <c r="O6" s="10"/>
-      <c r="T6" s="1"/>
-    </row>
-    <row r="7" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L6" s="10"/>
+      <c r="Q6" s="1"/>
+    </row>
+    <row r="7" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>17</v>
       </c>
@@ -1333,74 +1328,73 @@
         <f>SUM(F3:F6)</f>
         <v>79.616666666666674</v>
       </c>
-      <c r="J7">
+      <c r="G7">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K7" s="9" t="s">
+      <c r="H7" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="L7" s="7">
+      <c r="I7" s="7">
         <v>150</v>
       </c>
-      <c r="M7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="N7" s="8">
+      <c r="J7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" s="8">
         <v>18.5</v>
       </c>
-      <c r="O7" s="10"/>
-      <c r="T7" s="1"/>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="L7" s="10"/>
+      <c r="Q7" s="1"/>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F8" s="2"/>
-      <c r="H8" s="1"/>
-      <c r="J8">
+      <c r="G8">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="K8" s="9" t="s">
+      <c r="H8" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="L8" s="7">
+      <c r="I8" s="7">
         <v>24</v>
       </c>
-      <c r="M8" s="7" t="s">
+      <c r="J8" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="N8" s="8">
+      <c r="K8" s="8">
         <v>37</v>
       </c>
-      <c r="O8" s="10"/>
-      <c r="P8" t="s">
+      <c r="L8" s="10"/>
+      <c r="M8" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="49"/>
       <c r="B9" s="49"/>
-      <c r="J9">
+      <c r="G9">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="K9" s="9" t="s">
+      <c r="H9" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="L9" s="7">
+      <c r="I9" s="7">
         <v>432</v>
       </c>
-      <c r="M9" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="N9" s="8">
+      <c r="J9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K9" s="8">
         <v>38</v>
       </c>
-      <c r="O9" s="10"/>
-      <c r="P9" t="s">
+      <c r="L9" s="10"/>
+      <c r="M9" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:17" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A10" s="46" t="s">
         <v>58</v>
       </c>
@@ -1409,26 +1403,25 @@
       <c r="D10" s="47"/>
       <c r="E10" s="47"/>
       <c r="F10" s="48"/>
-      <c r="G10" s="1"/>
-      <c r="J10">
+      <c r="G10">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="K10" s="9" t="s">
+      <c r="H10" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="L10" s="7">
-        <v>13</v>
-      </c>
-      <c r="M10" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="N10" s="8">
+      <c r="I10" s="7">
+        <v>13</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K10" s="8">
         <v>6.5</v>
       </c>
-      <c r="O10" s="10"/>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="L10" s="10"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="22" t="s">
         <v>49</v>
       </c>
@@ -1447,27 +1440,27 @@
       <c r="F11" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="J11">
+      <c r="G11">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="H11" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="L11" s="7">
-        <v>13</v>
-      </c>
-      <c r="M11" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="N11" s="8">
+      <c r="I11" s="7">
+        <v>13</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K11" s="8">
         <v>5.8</v>
       </c>
-      <c r="O11" s="10"/>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="L11" s="10"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="str">
-        <f>K6</f>
+        <f>H6</f>
         <v>Ciruela cocida</v>
       </c>
       <c r="B12" s="27">
@@ -1480,34 +1473,34 @@
         <v>52</v>
       </c>
       <c r="E12" s="21">
-        <f>N6</f>
+        <f>K6</f>
         <v>60</v>
       </c>
       <c r="F12" s="24">
         <f>E12*B12</f>
         <v>60</v>
       </c>
-      <c r="J12">
+      <c r="G12">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="K12" s="9" t="s">
+      <c r="H12" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L12" s="7">
-        <v>13</v>
-      </c>
-      <c r="M12" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="N12" s="8">
+      <c r="I12" s="7">
+        <v>13</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K12" s="8">
         <v>5.8</v>
       </c>
-      <c r="O12" s="10"/>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="L12" s="10"/>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="str">
-        <f>K5</f>
+        <f>H5</f>
         <v>Leche condensada</v>
       </c>
       <c r="B13" s="27">
@@ -1517,36 +1510,36 @@
         <v>380</v>
       </c>
       <c r="D13" s="7" t="str">
-        <f>M5</f>
+        <f>J5</f>
         <v>grs</v>
       </c>
       <c r="E13" s="21">
-        <f>N5</f>
+        <f>K5</f>
         <v>29</v>
       </c>
       <c r="F13" s="24">
         <f>E13*B13</f>
         <v>14.5</v>
       </c>
-      <c r="J13">
+      <c r="G13">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="K13" s="9" t="s">
+      <c r="H13" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="L13" s="7">
+      <c r="I13" s="7">
         <v>255</v>
       </c>
-      <c r="M13" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="N13" s="8">
+      <c r="J13" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K13" s="8">
         <v>56</v>
       </c>
-      <c r="O13" s="10"/>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="L13" s="10"/>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="str">
         <f>$A$1</f>
         <v>Preparacion base de leche</v>
@@ -1569,25 +1562,25 @@
         <f>$F$7</f>
         <v>79.616666666666674</v>
       </c>
-      <c r="J14">
+      <c r="G14">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="K14" s="9" t="s">
+      <c r="H14" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="L14" s="7">
+      <c r="I14" s="7">
         <v>1</v>
       </c>
-      <c r="M14" s="7" t="s">
+      <c r="J14" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="N14" s="8">
+      <c r="K14" s="8">
         <v>20</v>
       </c>
-      <c r="O14" s="10"/>
-    </row>
-    <row r="15" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L14" s="10"/>
+    </row>
+    <row r="15" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
         <v>47</v>
       </c>
@@ -1601,32 +1594,32 @@
         <v>13</v>
       </c>
       <c r="E15" s="25">
-        <f xml:space="preserve"> $N$22 / 1000 * 11.7</f>
+        <f xml:space="preserve"> $K$22 / 1000 * 11.7</f>
         <v>1.3922999999999999</v>
       </c>
       <c r="F15" s="26">
         <f>E15*C15</f>
         <v>16.289909999999999</v>
       </c>
-      <c r="J15">
+      <c r="G15">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="K15" s="9" t="s">
+      <c r="H15" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="L15" s="7">
+      <c r="I15" s="7">
         <v>2</v>
       </c>
-      <c r="M15" s="7" t="s">
+      <c r="J15" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="N15" s="8">
+      <c r="K15" s="8">
         <v>183</v>
       </c>
-      <c r="O15" s="10"/>
-    </row>
-    <row r="16" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L15" s="10"/>
+    </row>
+    <row r="16" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
@@ -1638,25 +1631,25 @@
         <f>SUM(F12:F15)</f>
         <v>170.40657666666667</v>
       </c>
-      <c r="J16">
+      <c r="G16">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="K16" s="9" t="s">
+      <c r="H16" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="L16" s="7">
+      <c r="I16" s="7">
         <v>47</v>
       </c>
-      <c r="M16" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="N16" s="8">
+      <c r="J16" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K16" s="8">
         <v>14.2</v>
       </c>
-      <c r="O16" s="10"/>
-    </row>
-    <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L16" s="10"/>
+    </row>
+    <row r="17" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>51</v>
       </c>
@@ -1668,25 +1661,25 @@
         <f>B15</f>
         <v>14</v>
       </c>
-      <c r="J17">
+      <c r="G17">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="K17" s="9" t="s">
+      <c r="H17" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="L17" s="7">
+      <c r="I17" s="7">
         <v>47</v>
       </c>
-      <c r="M17" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="N17" s="8">
+      <c r="J17" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K17" s="8">
         <v>14.3</v>
       </c>
-      <c r="O17" s="10"/>
-    </row>
-    <row r="18" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L17" s="10"/>
+    </row>
+    <row r="18" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>4</v>
       </c>
@@ -1698,85 +1691,84 @@
         <v>5</v>
       </c>
       <c r="D18" s="6">
-        <f>$L$26</f>
-        <v>25</v>
+        <f>$I$26</f>
+        <v>30</v>
       </c>
       <c r="E18" s="31" t="s">
         <v>6</v>
       </c>
       <c r="F18" s="5">
         <f>D18-B18</f>
-        <v>12.828101666666667</v>
-      </c>
-      <c r="G18" s="37"/>
-      <c r="J18">
+        <v>17.828101666666669</v>
+      </c>
+      <c r="G18">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="K18" s="9" t="s">
+      <c r="H18" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="L18" s="7">
+      <c r="I18" s="7">
         <v>1</v>
       </c>
-      <c r="M18" s="7" t="s">
+      <c r="J18" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="N18" s="8">
+      <c r="K18" s="8">
         <v>577</v>
       </c>
-      <c r="O18" s="10"/>
-    </row>
-    <row r="19" spans="1:15" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="38" t="s">
+      <c r="L18" s="10"/>
+    </row>
+    <row r="19" spans="1:12" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="B19" s="39"/>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="40">
+      <c r="B19" s="38"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="38"/>
+      <c r="F19" s="39">
         <f>((D18-B18)/D18)</f>
-        <v>0.51312406666666666</v>
-      </c>
-      <c r="J19">
+        <v>0.59427005555555568</v>
+      </c>
+      <c r="G19">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="K19" s="9" t="s">
+      <c r="H19" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="L19" s="7">
+      <c r="I19" s="7">
         <v>100</v>
       </c>
-      <c r="M19" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="N19" s="8">
+      <c r="J19" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K19" s="8">
         <v>25</v>
       </c>
-      <c r="O19" s="10"/>
-    </row>
-    <row r="20" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="J20">
+      <c r="L19" s="10"/>
+    </row>
+    <row r="20" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G20">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="K20" s="9" t="s">
+      <c r="H20" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="L20" s="7">
+      <c r="I20" s="7">
         <v>1</v>
       </c>
-      <c r="M20" s="7" t="s">
+      <c r="J20" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="N20" s="8">
+      <c r="K20" s="8">
         <v>24</v>
       </c>
-      <c r="O20" s="10"/>
-    </row>
-    <row r="21" spans="1:15" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="L20" s="10"/>
+    </row>
+    <row r="21" spans="1:12" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A21" s="46" t="s">
         <v>59</v>
       </c>
@@ -1785,25 +1777,25 @@
       <c r="D21" s="47"/>
       <c r="E21" s="47"/>
       <c r="F21" s="48"/>
-      <c r="J21">
+      <c r="G21">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="K21" s="9" t="s">
+      <c r="H21" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="L21" s="7">
+      <c r="I21" s="7">
         <v>120</v>
       </c>
-      <c r="M21" s="7" t="s">
+      <c r="J21" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="N21" s="8">
+      <c r="K21" s="8">
         <v>44</v>
       </c>
-      <c r="O21" s="10"/>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L21" s="10"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="22" t="s">
         <v>49</v>
       </c>
@@ -1822,28 +1814,27 @@
       <c r="F22" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="H22" s="2"/>
-      <c r="J22">
+      <c r="G22">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="K22" s="53" t="s">
+      <c r="H22" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="L22" s="7">
+      <c r="I22" s="7">
         <v>1</v>
       </c>
-      <c r="M22" s="7" t="s">
+      <c r="J22" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="N22" s="8">
+      <c r="K22" s="8">
         <v>119</v>
       </c>
-      <c r="O22" s="10"/>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L22" s="10"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="str">
-        <f>K15</f>
+        <f>H15</f>
         <v>Fresas congelada</v>
       </c>
       <c r="B23" s="27">
@@ -1862,27 +1853,27 @@
         <f>E23*B23</f>
         <v>16</v>
       </c>
-      <c r="J23">
+      <c r="G23">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="K23" s="9" t="s">
+      <c r="H23" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="L23" s="7">
+      <c r="I23" s="7">
         <v>500</v>
       </c>
-      <c r="M23" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="N23" s="8">
+      <c r="J23" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K23" s="8">
         <v>60</v>
       </c>
-      <c r="O23" s="10"/>
-    </row>
-    <row r="24" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L23" s="10"/>
+    </row>
+    <row r="24" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="str">
-        <f>K12</f>
+        <f>H12</f>
         <v>Sobre de tang fresa</v>
       </c>
       <c r="B24" s="27">
@@ -1895,32 +1886,32 @@
         <v>13</v>
       </c>
       <c r="E24" s="21">
-        <f>N12</f>
+        <f>K12</f>
         <v>5.8</v>
       </c>
       <c r="F24" s="24">
         <f>E24*B24</f>
         <v>5.8</v>
       </c>
-      <c r="J24">
+      <c r="G24">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="K24" s="12" t="s">
+      <c r="H24" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="L24" s="13">
+      <c r="I24" s="13">
         <v>1</v>
       </c>
-      <c r="M24" s="13" t="s">
+      <c r="J24" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="N24" s="14">
+      <c r="K24" s="14">
         <v>25</v>
       </c>
-      <c r="O24" s="15"/>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L24" s="15"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="str">
         <f>$A$1</f>
         <v>Preparacion base de leche</v>
@@ -1944,7 +1935,7 @@
         <v>79.616666666666674</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
         <v>47</v>
       </c>
@@ -1958,21 +1949,21 @@
         <v>13</v>
       </c>
       <c r="E26" s="25">
-        <f xml:space="preserve"> $N$22 / 1000 * 11.7</f>
+        <f xml:space="preserve"> $K$22 / 1000 * 11.7</f>
         <v>1.3922999999999999</v>
       </c>
       <c r="F26" s="26">
         <f>E26*C26</f>
         <v>16.289909999999999</v>
       </c>
-      <c r="K26" t="s">
+      <c r="H26" t="s">
         <v>63</v>
       </c>
-      <c r="L26" s="1">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I26" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>17</v>
       </c>
@@ -1984,14 +1975,14 @@
         <f>SUM(F23:F26)</f>
         <v>117.70657666666668</v>
       </c>
-      <c r="K27" t="s">
+      <c r="H27" t="s">
         <v>68</v>
       </c>
-      <c r="L27" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I27" s="1">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>51</v>
       </c>
@@ -2003,15 +1994,14 @@
         <f>B26</f>
         <v>12</v>
       </c>
-      <c r="G28" s="37"/>
-      <c r="K28" t="s">
+      <c r="H28" t="s">
         <v>69</v>
       </c>
-      <c r="L28" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I28" s="1">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>4</v>
       </c>
@@ -2023,35 +2013,34 @@
         <v>5</v>
       </c>
       <c r="D29" s="6">
-        <f>$L$26</f>
-        <v>25</v>
+        <f>$I$26</f>
+        <v>30</v>
       </c>
       <c r="E29" s="31" t="s">
         <v>6</v>
       </c>
       <c r="F29" s="5">
         <f>D29-B29</f>
-        <v>15.19111861111111</v>
-      </c>
-      <c r="G29" s="37"/>
-    </row>
-    <row r="30" spans="1:15" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="38" t="s">
+        <v>20.191118611111108</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="B30" s="39"/>
-      <c r="C30" s="39"/>
-      <c r="D30" s="39"/>
-      <c r="E30" s="39"/>
-      <c r="F30" s="40">
+      <c r="B30" s="38"/>
+      <c r="C30" s="38"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="38"/>
+      <c r="F30" s="39">
         <f>((D29-B29)/D29)</f>
-        <v>0.60764474444444438</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0.67303728703703691</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="30"/>
     </row>
-    <row r="32" spans="1:15" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:12" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A32" s="46" t="s">
         <v>53</v>
       </c>
@@ -2061,7 +2050,7 @@
       <c r="E32" s="47"/>
       <c r="F32" s="48"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="22" t="s">
         <v>49</v>
       </c>
@@ -2081,9 +2070,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="str">
-        <f>$K$9</f>
+        <f>$H$9</f>
         <v>Galleta maria</v>
       </c>
       <c r="B34" s="27">
@@ -2096,7 +2085,7 @@
         <v>13</v>
       </c>
       <c r="E34" s="21">
-        <f>N9/3</f>
+        <f>K9/3</f>
         <v>12.666666666666666</v>
       </c>
       <c r="F34" s="24">
@@ -2104,7 +2093,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="str">
         <f>$A$1</f>
         <v>Preparacion base de leche</v>
@@ -2128,7 +2117,7 @@
         <v>79.616666666666674</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="12" t="s">
         <v>47</v>
       </c>
@@ -2142,7 +2131,7 @@
         <v>13</v>
       </c>
       <c r="E36" s="25">
-        <f xml:space="preserve"> $N$22 / 1000 * 11.7</f>
+        <f xml:space="preserve"> $K$22 / 1000 * 11.7</f>
         <v>1.3922999999999999</v>
       </c>
       <c r="F36" s="26">
@@ -2150,7 +2139,7 @@
         <v>16.289909999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>17</v>
       </c>
@@ -2163,7 +2152,7 @@
         <v>114.90657666666667</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
         <v>51</v>
       </c>
@@ -2175,9 +2164,8 @@
         <f>B36</f>
         <v>12</v>
       </c>
-      <c r="G38" s="37"/>
-    </row>
-    <row r="39" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
         <v>4</v>
       </c>
@@ -2189,33 +2177,32 @@
         <v>5</v>
       </c>
       <c r="D39" s="6">
-        <f>$L$26</f>
-        <v>25</v>
+        <f>$I$26</f>
+        <v>30</v>
       </c>
       <c r="E39" s="31" t="s">
         <v>6</v>
       </c>
       <c r="F39" s="5">
         <f>D39-B39</f>
-        <v>15.424451944444444</v>
-      </c>
-      <c r="G39" s="37"/>
-    </row>
-    <row r="40" spans="1:7" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A40" s="38" t="s">
+        <v>20.424451944444442</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A40" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="B40" s="39"/>
-      <c r="C40" s="39"/>
-      <c r="D40" s="39"/>
-      <c r="E40" s="39"/>
-      <c r="F40" s="40">
+      <c r="B40" s="38"/>
+      <c r="C40" s="38"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="38"/>
+      <c r="F40" s="39">
         <f>((D39-B39)/D39)</f>
-        <v>0.6169780777777778</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="42" spans="1:7" ht="26.25" x14ac:dyDescent="0.4">
+        <v>0.68081506481481469</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="42" spans="1:6" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A42" s="46" t="s">
         <v>60</v>
       </c>
@@ -2225,7 +2212,7 @@
       <c r="E42" s="47"/>
       <c r="F42" s="48"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="22" t="s">
         <v>49</v>
       </c>
@@ -2245,9 +2232,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="str">
-        <f>K8</f>
+        <f>H8</f>
         <v>Galleta oreo</v>
       </c>
       <c r="B44" s="27">
@@ -2260,7 +2247,7 @@
         <v>13</v>
       </c>
       <c r="E44" s="21">
-        <f>N9/24</f>
+        <f>K9/24</f>
         <v>1.5833333333333333</v>
       </c>
       <c r="F44" s="24">
@@ -2268,7 +2255,7 @@
         <v>20.583333333333332</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="str">
         <f>$A$1</f>
         <v>Preparacion base de leche</v>
@@ -2292,7 +2279,7 @@
         <v>79.616666666666674</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="12" t="s">
         <v>47</v>
       </c>
@@ -2306,7 +2293,7 @@
         <v>13</v>
       </c>
       <c r="E46" s="25">
-        <f xml:space="preserve"> $N$22 / 1000 * 11.7</f>
+        <f xml:space="preserve"> $K$22 / 1000 * 11.7</f>
         <v>1.3922999999999999</v>
       </c>
       <c r="F46" s="26">
@@ -2314,7 +2301,7 @@
         <v>16.289909999999999</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>17</v>
       </c>
@@ -2327,7 +2314,7 @@
         <v>116.48991000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>51</v>
       </c>
@@ -2339,9 +2326,8 @@
         <f>B46</f>
         <v>12</v>
       </c>
-      <c r="G48" s="37"/>
-    </row>
-    <row r="49" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="49" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
         <v>4</v>
       </c>
@@ -2353,35 +2339,33 @@
         <v>5</v>
       </c>
       <c r="D49" s="6">
-        <f>$L$26</f>
-        <v>25</v>
+        <f>$I$26</f>
+        <v>30</v>
       </c>
       <c r="E49" s="31" t="s">
         <v>6</v>
       </c>
       <c r="F49" s="5">
         <f>D49-B49</f>
-        <v>15.292507499999999</v>
-      </c>
-      <c r="G49" s="37"/>
-    </row>
-    <row r="50" spans="1:10" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A50" s="38" t="s">
+        <v>20.292507499999999</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A50" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="B50" s="39"/>
-      <c r="C50" s="39"/>
-      <c r="D50" s="39"/>
-      <c r="E50" s="39"/>
-      <c r="F50" s="40">
+      <c r="B50" s="38"/>
+      <c r="C50" s="38"/>
+      <c r="D50" s="38"/>
+      <c r="E50" s="38"/>
+      <c r="F50" s="39">
         <f>((D49-B49)/D49)</f>
-        <v>0.61170029999999997</v>
-      </c>
-      <c r="I50" s="2"/>
-      <c r="J50" s="2"/>
-    </row>
-    <row r="51" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="52" spans="1:10" ht="26.25" x14ac:dyDescent="0.4">
+        <v>0.67641691666666659</v>
+      </c>
+      <c r="G50" s="2"/>
+    </row>
+    <row r="51" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="52" spans="1:7" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A52" s="46" t="s">
         <v>1</v>
       </c>
@@ -2391,7 +2375,7 @@
       <c r="E52" s="47"/>
       <c r="F52" s="48"/>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="22" t="s">
         <v>49</v>
       </c>
@@ -2411,9 +2395,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="str">
-        <f>K16</f>
+        <f>H16</f>
         <v>Maicena nuez</v>
       </c>
       <c r="B54" s="27">
@@ -2426,7 +2410,7 @@
         <v>13</v>
       </c>
       <c r="E54" s="21">
-        <f>N16</f>
+        <f>K16</f>
         <v>14.2</v>
       </c>
       <c r="F54" s="24">
@@ -2434,7 +2418,7 @@
         <v>14.2</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="str">
         <f>$A$1</f>
         <v>Preparacion base de leche</v>
@@ -2458,7 +2442,7 @@
         <v>79.616666666666674</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="12" t="s">
         <v>47</v>
       </c>
@@ -2472,7 +2456,7 @@
         <v>13</v>
       </c>
       <c r="E56" s="25">
-        <f xml:space="preserve"> $N$22 / 1000 * 11.7</f>
+        <f xml:space="preserve"> $K$22 / 1000 * 11.7</f>
         <v>1.3922999999999999</v>
       </c>
       <c r="F56" s="26">
@@ -2480,7 +2464,7 @@
         <v>16.289909999999999</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
         <v>17</v>
       </c>
@@ -2493,7 +2477,7 @@
         <v>110.10657666666668</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
         <v>51</v>
       </c>
@@ -2505,9 +2489,8 @@
         <f>B56</f>
         <v>12</v>
       </c>
-      <c r="G58" s="37"/>
-    </row>
-    <row r="59" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="59" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
         <v>4</v>
       </c>
@@ -2519,33 +2502,32 @@
         <v>5</v>
       </c>
       <c r="D59" s="6">
-        <f>$L$26</f>
-        <v>25</v>
+        <f>$I$26</f>
+        <v>30</v>
       </c>
       <c r="E59" s="31" t="s">
         <v>6</v>
       </c>
       <c r="F59" s="5">
         <f>D59-B59</f>
-        <v>15.824451944444442</v>
-      </c>
-      <c r="G59" s="37"/>
-    </row>
-    <row r="60" spans="1:10" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A60" s="38" t="s">
+        <v>20.824451944444441</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A60" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="B60" s="39"/>
-      <c r="C60" s="39"/>
-      <c r="D60" s="39"/>
-      <c r="E60" s="39"/>
-      <c r="F60" s="40">
+      <c r="B60" s="38"/>
+      <c r="C60" s="38"/>
+      <c r="D60" s="38"/>
+      <c r="E60" s="38"/>
+      <c r="F60" s="39">
         <f>((D59-B59)/D59)</f>
-        <v>0.6329780777777777</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="62" spans="1:10" ht="26.25" x14ac:dyDescent="0.4">
+        <v>0.69414839814814799</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="62" spans="1:7" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A62" s="46" t="s">
         <v>9</v>
       </c>
@@ -2555,7 +2537,7 @@
       <c r="E62" s="47"/>
       <c r="F62" s="48"/>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="22" t="s">
         <v>49</v>
       </c>
@@ -2575,23 +2557,23 @@
         <v>50</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="9" t="str">
-        <f>K17</f>
+        <f>H17</f>
         <v>Maicena coco</v>
       </c>
       <c r="B64" s="27">
         <v>1</v>
       </c>
       <c r="C64" s="7">
-        <f>L17</f>
+        <f>I17</f>
         <v>47</v>
       </c>
       <c r="D64" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E64" s="21">
-        <f>N17</f>
+        <f>K17</f>
         <v>14.3</v>
       </c>
       <c r="F64" s="24">
@@ -2599,7 +2581,7 @@
         <v>14.3</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="9" t="str">
         <f>$A$1</f>
         <v>Preparacion base de leche</v>
@@ -2623,7 +2605,7 @@
         <v>79.616666666666674</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="12" t="s">
         <v>47</v>
       </c>
@@ -2637,7 +2619,7 @@
         <v>13</v>
       </c>
       <c r="E66" s="25">
-        <f xml:space="preserve"> $N$22 / 1000 * 11.7</f>
+        <f xml:space="preserve"> $K$22 / 1000 * 11.7</f>
         <v>1.3922999999999999</v>
       </c>
       <c r="F66" s="26">
@@ -2645,7 +2627,7 @@
         <v>16.289909999999999</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
         <v>17</v>
       </c>
@@ -2658,7 +2640,7 @@
         <v>110.20657666666668</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
         <v>51</v>
       </c>
@@ -2670,9 +2652,8 @@
         <f>B66</f>
         <v>12</v>
       </c>
-      <c r="G68" s="37"/>
-    </row>
-    <row r="69" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="69" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
         <v>4</v>
       </c>
@@ -2684,33 +2665,32 @@
         <v>5</v>
       </c>
       <c r="D69" s="6">
-        <f>$L$26</f>
-        <v>25</v>
+        <f>$I$26</f>
+        <v>30</v>
       </c>
       <c r="E69" s="31" t="s">
         <v>6</v>
       </c>
       <c r="F69" s="5">
         <f>D69-B69</f>
-        <v>15.81611861111111</v>
-      </c>
-      <c r="G69" s="37"/>
-    </row>
-    <row r="70" spans="1:11" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A70" s="38" t="s">
+        <v>20.816118611111108</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A70" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="B70" s="39"/>
-      <c r="C70" s="39"/>
-      <c r="D70" s="39"/>
-      <c r="E70" s="39"/>
-      <c r="F70" s="40">
+      <c r="B70" s="38"/>
+      <c r="C70" s="38"/>
+      <c r="D70" s="38"/>
+      <c r="E70" s="38"/>
+      <c r="F70" s="39">
         <f>((D69-B69)/D69)</f>
-        <v>0.63264474444444441</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="72" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
+        <v>0.69387062037037028</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="72" spans="1:8" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A72" s="46" t="s">
         <v>2</v>
       </c>
@@ -2720,7 +2700,7 @@
       <c r="E72" s="47"/>
       <c r="F72" s="48"/>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="22" t="s">
         <v>49</v>
       </c>
@@ -2740,9 +2720,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="9" t="str">
-        <f>K21</f>
+        <f>H21</f>
         <v>Vainilla para helados</v>
       </c>
       <c r="B74" s="27">
@@ -2755,7 +2735,7 @@
         <v>61</v>
       </c>
       <c r="E74" s="21">
-        <f>N21/4</f>
+        <f>K21/4</f>
         <v>11</v>
       </c>
       <c r="F74" s="24">
@@ -2763,7 +2743,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="9" t="str">
         <f>$A$1</f>
         <v>Preparacion base de leche</v>
@@ -2787,7 +2767,7 @@
         <v>79.616666666666674</v>
       </c>
     </row>
-    <row r="76" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="12" t="s">
         <v>47</v>
       </c>
@@ -2801,7 +2781,7 @@
         <v>13</v>
       </c>
       <c r="E76" s="25">
-        <f xml:space="preserve"> $N$22 / 1000 * 11.7</f>
+        <f xml:space="preserve"> $K$22 / 1000 * 11.7</f>
         <v>1.3922999999999999</v>
       </c>
       <c r="F76" s="26">
@@ -2809,7 +2789,7 @@
         <v>16.289909999999999</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="3" t="s">
         <v>17</v>
       </c>
@@ -2822,7 +2802,7 @@
         <v>106.90657666666667</v>
       </c>
     </row>
-    <row r="78" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="3" t="s">
         <v>51</v>
       </c>
@@ -2834,9 +2814,8 @@
         <f>B76</f>
         <v>12</v>
       </c>
-      <c r="G78" s="37"/>
-    </row>
-    <row r="79" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="79" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="3" t="s">
         <v>4</v>
       </c>
@@ -2848,29 +2827,29 @@
         <v>5</v>
       </c>
       <c r="D79" s="6">
-        <f>$L$26</f>
-        <v>25</v>
+        <f>$I$26</f>
+        <v>30</v>
       </c>
       <c r="E79" s="31" t="s">
         <v>6</v>
       </c>
       <c r="F79" s="5">
         <f>D79-B79</f>
-        <v>16.091118611111114</v>
-      </c>
-      <c r="K79" s="1"/>
-    </row>
-    <row r="80" spans="1:11" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A80" s="38" t="s">
+        <v>21.091118611111114</v>
+      </c>
+      <c r="H79" s="1"/>
+    </row>
+    <row r="80" spans="1:8" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A80" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="B80" s="39"/>
-      <c r="C80" s="39"/>
-      <c r="D80" s="39"/>
-      <c r="E80" s="39"/>
-      <c r="F80" s="40">
+      <c r="B80" s="38"/>
+      <c r="C80" s="38"/>
+      <c r="D80" s="38"/>
+      <c r="E80" s="38"/>
+      <c r="F80" s="39">
         <f>((D79-B79)/D79)</f>
-        <v>0.64364474444444453</v>
+        <v>0.70303728703703716</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -2906,7 +2885,7 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="9" t="str">
-        <f>K18</f>
+        <f>H18</f>
         <v>Baileys</v>
       </c>
       <c r="B84" s="27">
@@ -2919,7 +2898,7 @@
         <v>42</v>
       </c>
       <c r="E84" s="21">
-        <f>N18</f>
+        <f>K18</f>
         <v>577</v>
       </c>
       <c r="F84" s="24">
@@ -2965,7 +2944,7 @@
         <v>13</v>
       </c>
       <c r="E86" s="25">
-        <f xml:space="preserve"> $N$22 / 1000 * 11.7</f>
+        <f xml:space="preserve"> $K$22 / 1000 * 11.7</f>
         <v>1.3922999999999999</v>
       </c>
       <c r="F86" s="26">
@@ -3011,28 +2990,28 @@
         <v>5</v>
       </c>
       <c r="D89" s="6">
-        <f>$L$27</f>
-        <v>30</v>
+        <f>$I$27</f>
+        <v>35</v>
       </c>
       <c r="E89" s="31" t="s">
         <v>6</v>
       </c>
       <c r="F89" s="5">
         <f>D89-B89</f>
-        <v>9.9869519444444457</v>
+        <v>14.986951944444446</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A90" s="38" t="s">
+      <c r="A90" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="B90" s="39"/>
-      <c r="C90" s="39"/>
-      <c r="D90" s="39"/>
-      <c r="E90" s="39"/>
-      <c r="F90" s="40">
+      <c r="B90" s="38"/>
+      <c r="C90" s="38"/>
+      <c r="D90" s="38"/>
+      <c r="E90" s="38"/>
+      <c r="F90" s="39">
         <f>((D89-B89)/D89)</f>
-        <v>0.3328983981481482</v>
+        <v>0.42819862698412703</v>
       </c>
     </row>
     <row r="91" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -3068,7 +3047,7 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="9" t="str">
-        <f>$K$20</f>
+        <f>$H$20</f>
         <v>Azúcar</v>
       </c>
       <c r="B94" s="27">
@@ -3126,7 +3105,7 @@
         <v>13</v>
       </c>
       <c r="E96" s="25">
-        <f xml:space="preserve"> $N$22 / 1000 * 11.7</f>
+        <f xml:space="preserve"> $K$22 / 1000 * 11.7</f>
         <v>1.3922999999999999</v>
       </c>
       <c r="F96" s="26">
@@ -3134,7 +3113,7 @@
         <v>16.289909999999999</v>
       </c>
     </row>
-    <row r="97" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A97" s="3" t="s">
         <v>17</v>
       </c>
@@ -3147,7 +3126,7 @@
         <v>104.18657666666667</v>
       </c>
     </row>
-    <row r="98" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
         <v>51</v>
       </c>
@@ -3160,7 +3139,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="99" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" s="3" t="s">
         <v>4</v>
       </c>
@@ -3172,32 +3151,32 @@
         <v>5</v>
       </c>
       <c r="D99" s="6">
-        <f>$L$26</f>
-        <v>25</v>
+        <f>$I$26</f>
+        <v>30</v>
       </c>
       <c r="E99" s="31" t="s">
         <v>6</v>
       </c>
       <c r="F99" s="5">
         <f>D99-B99</f>
-        <v>16.31778527777778</v>
-      </c>
-    </row>
-    <row r="100" spans="1:11" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A100" s="38" t="s">
+        <v>21.31778527777778</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A100" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="B100" s="39"/>
-      <c r="C100" s="39"/>
-      <c r="D100" s="39"/>
-      <c r="E100" s="39"/>
-      <c r="F100" s="40">
+      <c r="B100" s="38"/>
+      <c r="C100" s="38"/>
+      <c r="D100" s="38"/>
+      <c r="E100" s="38"/>
+      <c r="F100" s="39">
         <f>((D99-B99)/D99)</f>
-        <v>0.65271141111111119</v>
-      </c>
-    </row>
-    <row r="101" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="102" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
+        <v>0.7105928425925927</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="102" spans="1:8" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A102" s="46" t="s">
         <v>65</v>
       </c>
@@ -3207,30 +3186,30 @@
       <c r="E102" s="47"/>
       <c r="F102" s="48"/>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="B103" s="43" t="s">
+      <c r="B103" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="C103" s="43" t="s">
+      <c r="C103" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="D103" s="43" t="s">
+      <c r="D103" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="E103" s="43" t="s">
+      <c r="E103" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="F103" s="44" t="s">
+      <c r="F103" s="43" t="s">
         <v>50</v>
       </c>
-      <c r="K103" s="1"/>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H103" s="1"/>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" s="9" t="str">
-        <f>$K$20</f>
+        <f>$H$20</f>
         <v>Azúcar</v>
       </c>
       <c r="B104" s="27">
@@ -3249,11 +3228,11 @@
         <f>(E104/C104)*B104</f>
         <v>8.2799999999999994</v>
       </c>
-      <c r="K104" s="1"/>
-    </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H104" s="1"/>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" s="9" t="str">
-        <f>K14</f>
+        <f>H14</f>
         <v>Mango</v>
       </c>
       <c r="B105" s="27">
@@ -3266,32 +3245,32 @@
         <v>13</v>
       </c>
       <c r="E105" s="21">
-        <f>N14</f>
+        <f>K14</f>
         <v>20</v>
       </c>
       <c r="F105" s="24">
         <f>(E105/C105)*B105</f>
         <v>10</v>
       </c>
-      <c r="K105" s="1"/>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H105" s="1"/>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" s="32" t="str">
-        <f>K11</f>
+        <f>H11</f>
         <v>Sobre de tang mango</v>
       </c>
       <c r="B106" s="33">
         <v>6.5</v>
       </c>
       <c r="C106" s="34">
-        <f>L11</f>
+        <f>I11</f>
         <v>13</v>
       </c>
       <c r="D106" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E106" s="41">
-        <f>N11</f>
+      <c r="E106" s="40">
+        <f>K11</f>
         <v>5.8</v>
       </c>
       <c r="F106" s="24">
@@ -3299,23 +3278,23 @@
         <v>2.9</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" s="32" t="str">
-        <f>K13</f>
+        <f>H13</f>
         <v>Tajin</v>
       </c>
       <c r="B107" s="33">
         <v>30</v>
       </c>
       <c r="C107" s="34">
-        <f>L13</f>
+        <f>I13</f>
         <v>255</v>
       </c>
       <c r="D107" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E107" s="41">
-        <f>N13</f>
+      <c r="E107" s="40">
+        <f>K13</f>
         <v>56</v>
       </c>
       <c r="F107" s="24">
@@ -3323,23 +3302,23 @@
         <v>6.5882352941176467</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" s="9" t="str">
-        <f>$K$4</f>
+        <f>$H$4</f>
         <v>CMC</v>
       </c>
       <c r="B108" s="27">
         <v>7.5</v>
       </c>
       <c r="C108" s="7">
-        <f>L4</f>
+        <f>I4</f>
         <v>180</v>
       </c>
       <c r="D108" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E108" s="21">
-        <f>N4</f>
+        <f>K4</f>
         <v>58</v>
       </c>
       <c r="F108" s="24">
@@ -3347,27 +3326,27 @@
         <v>2.416666666666667</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" s="32" t="s">
         <v>0</v>
       </c>
       <c r="B109" s="33">
         <v>1500</v>
       </c>
-      <c r="C109" s="45">
+      <c r="C109" s="44">
         <v>1.5</v>
       </c>
       <c r="D109" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="E109" s="41">
+      <c r="E109" s="40">
         <v>5</v>
       </c>
-      <c r="F109" s="42">
+      <c r="F109" s="41">
         <v>5</v>
       </c>
     </row>
-    <row r="110" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A110" s="12" t="s">
         <v>47</v>
       </c>
@@ -3381,7 +3360,7 @@
         <v>13</v>
       </c>
       <c r="E110" s="25">
-        <f xml:space="preserve"> $N$22 / 1000 * 11.7</f>
+        <f xml:space="preserve"> $K$22 / 1000 * 11.7</f>
         <v>1.3922999999999999</v>
       </c>
       <c r="F110" s="26">
@@ -3389,7 +3368,7 @@
         <v>16.289909999999999</v>
       </c>
     </row>
-    <row r="111" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A111" s="3" t="s">
         <v>17</v>
       </c>
@@ -3402,7 +3381,7 @@
         <v>51.474811960784315</v>
       </c>
     </row>
-    <row r="112" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A112" s="3" t="s">
         <v>51</v>
       </c>
@@ -3427,28 +3406,28 @@
         <v>5</v>
       </c>
       <c r="D113" s="6">
-        <f>$L$28</f>
-        <v>20</v>
+        <f>$I$28</f>
+        <v>25</v>
       </c>
       <c r="E113" s="31" t="s">
         <v>6</v>
       </c>
       <c r="F113" s="5">
         <f>D113-B113</f>
-        <v>16.323227717086834</v>
+        <v>21.323227717086834</v>
       </c>
     </row>
     <row r="114" spans="1:6" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A114" s="38" t="s">
+      <c r="A114" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="B114" s="39"/>
-      <c r="C114" s="39"/>
-      <c r="D114" s="39"/>
-      <c r="E114" s="39"/>
-      <c r="F114" s="40">
+      <c r="B114" s="38"/>
+      <c r="C114" s="38"/>
+      <c r="D114" s="38"/>
+      <c r="E114" s="38"/>
+      <c r="F114" s="39">
         <f>((D113-B113)/D113)</f>
-        <v>0.81616138585434173</v>
+        <v>0.85292910868347338</v>
       </c>
     </row>
     <row r="115" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -3466,38 +3445,38 @@
       <c r="A117" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="B117" s="43" t="s">
+      <c r="B117" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="C117" s="43" t="s">
+      <c r="C117" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="D117" s="43" t="s">
+      <c r="D117" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="E117" s="43" t="s">
+      <c r="E117" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="F117" s="44" t="s">
+      <c r="F117" s="43" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" s="32" t="str">
+        <f>H10</f>
+        <v>Sobre de tang limon</v>
+      </c>
+      <c r="B118" s="33">
+        <v>13</v>
+      </c>
+      <c r="C118" s="34">
+        <v>13</v>
+      </c>
+      <c r="D118" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E118" s="40">
         <f>K10</f>
-        <v>Sobre de tang limon</v>
-      </c>
-      <c r="B118" s="33">
-        <v>13</v>
-      </c>
-      <c r="C118" s="34">
-        <v>13</v>
-      </c>
-      <c r="D118" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E118" s="41">
-        <f>N10</f>
         <v>6.5</v>
       </c>
       <c r="F118" s="24">
@@ -3507,7 +3486,7 @@
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" s="9" t="str">
-        <f>$K$20</f>
+        <f>$H$20</f>
         <v>Azúcar</v>
       </c>
       <c r="B119" s="27">
@@ -3534,36 +3513,36 @@
       <c r="B120" s="33">
         <v>1500</v>
       </c>
-      <c r="C120" s="45">
+      <c r="C120" s="44">
         <v>1.5</v>
       </c>
       <c r="D120" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="E120" s="41">
+      <c r="E120" s="40">
         <v>5</v>
       </c>
-      <c r="F120" s="42">
+      <c r="F120" s="41">
         <v>5</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" s="9" t="str">
-        <f>$K$4</f>
+        <f>$H$4</f>
         <v>CMC</v>
       </c>
       <c r="B121" s="27">
         <v>7.5</v>
       </c>
       <c r="C121" s="7">
-        <f>L17</f>
+        <f>I17</f>
         <v>47</v>
       </c>
       <c r="D121" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E121" s="21">
-        <f>N17</f>
+        <f>K17</f>
         <v>14.3</v>
       </c>
       <c r="F121" s="24">
@@ -3585,7 +3564,7 @@
         <v>13</v>
       </c>
       <c r="E122" s="25">
-        <f xml:space="preserve"> $N$22 / 1000 * 11.7</f>
+        <f xml:space="preserve"> $K$22 / 1000 * 11.7</f>
         <v>1.3922999999999999</v>
       </c>
       <c r="F122" s="26">
@@ -3631,28 +3610,28 @@
         <v>5</v>
       </c>
       <c r="D125" s="6">
-        <f>$L$28</f>
-        <v>20</v>
+        <f>$I$28</f>
+        <v>25</v>
       </c>
       <c r="E125" s="31" t="s">
         <v>6</v>
       </c>
       <c r="F125" s="5">
         <f>D125-B125</f>
-        <v>17.560583936170215</v>
+        <v>22.560583936170215</v>
       </c>
     </row>
     <row r="126" spans="1:6" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A126" s="38" t="s">
+      <c r="A126" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="B126" s="39"/>
-      <c r="C126" s="39"/>
-      <c r="D126" s="39"/>
-      <c r="E126" s="39"/>
-      <c r="F126" s="40">
+      <c r="B126" s="38"/>
+      <c r="C126" s="38"/>
+      <c r="D126" s="38"/>
+      <c r="E126" s="38"/>
+      <c r="F126" s="39">
         <f>((D125-B125)/D125)</f>
-        <v>0.87802919680851077</v>
+        <v>0.90242335744680857</v>
       </c>
     </row>
     <row r="127" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -3688,7 +3667,7 @@
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" s="9" t="str">
-        <f>$K$9</f>
+        <f>$H$9</f>
         <v>Galleta maria</v>
       </c>
       <c r="B130" s="27">
@@ -3701,7 +3680,7 @@
         <v>13</v>
       </c>
       <c r="E130" s="21">
-        <f>N9/3</f>
+        <f>K9/3</f>
         <v>12.666666666666666</v>
       </c>
       <c r="F130" s="24">
@@ -3711,11 +3690,11 @@
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" s="9" t="str">
-        <f>K10</f>
+        <f>H10</f>
         <v>Sobre de tang limon</v>
       </c>
       <c r="B131" s="27">
-        <f>L10</f>
+        <f>I10</f>
         <v>13</v>
       </c>
       <c r="C131" s="7">
@@ -3725,8 +3704,8 @@
       <c r="D131" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E131" s="41">
-        <f>N10</f>
+      <c r="E131" s="40">
+        <f>K10</f>
         <v>6.5</v>
       </c>
       <c r="F131" s="24">
@@ -3772,7 +3751,7 @@
         <v>13</v>
       </c>
       <c r="E133" s="25">
-        <f xml:space="preserve"> $N$22 / 1000 * 11.7</f>
+        <f xml:space="preserve"> $K$22 / 1000 * 11.7</f>
         <v>1.3922999999999999</v>
       </c>
       <c r="F133" s="26">
@@ -3818,47 +3797,47 @@
         <v>5</v>
       </c>
       <c r="D136" s="6">
-        <f>$L$26</f>
-        <v>25</v>
+        <f>$I$26</f>
+        <v>30</v>
       </c>
       <c r="E136" s="31" t="s">
         <v>6</v>
       </c>
       <c r="F136" s="5">
         <f>D136-B136</f>
-        <v>15.938340833333333</v>
+        <v>20.938340833333335</v>
       </c>
     </row>
     <row r="137" spans="1:6" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A137" s="38" t="s">
+      <c r="A137" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="B137" s="39"/>
-      <c r="C137" s="39"/>
-      <c r="D137" s="39"/>
-      <c r="E137" s="39"/>
-      <c r="F137" s="40">
+      <c r="B137" s="38"/>
+      <c r="C137" s="38"/>
+      <c r="D137" s="38"/>
+      <c r="E137" s="38"/>
+      <c r="F137" s="39">
         <f>((D136-B136)/D136)</f>
-        <v>0.63753363333333335</v>
+        <v>0.69794469444444451</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A52:F52"/>
+    <mergeCell ref="A62:F62"/>
+    <mergeCell ref="A72:F72"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="H1:L1"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A21:F21"/>
     <mergeCell ref="A128:F128"/>
     <mergeCell ref="A82:F82"/>
     <mergeCell ref="A92:F92"/>
     <mergeCell ref="A102:F102"/>
     <mergeCell ref="A116:F116"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="K1:O1"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A42:F42"/>
-    <mergeCell ref="A52:F52"/>
-    <mergeCell ref="A62:F62"/>
-    <mergeCell ref="A72:F72"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>